<commit_message>
Use TFF for 超滤 in the project glossary and UF retrofit English files
The project term for 超滤 is TFF, not ultrafiltration or UF. Record it in the
CMC glossary and apply it to the English PPT and checklist.

Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/deliverables/超滤设备改造_EN.xlsx
+++ b/deliverables/超滤设备改造_EN.xlsx
@@ -326,7 +326,7 @@
         <rFont val="Times New Roman"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">UF</t>
+      <t xml:space="preserve">TFF</t>
     </r>
   </si>
   <si>
@@ -516,7 +516,7 @@
     <t>TFF</t>
   </si>
   <si>
-    <t xml:space="preserve">UF</t>
+    <t xml:space="preserve">TFF</t>
   </si>
   <si>
     <r>

</xml_diff>